<commit_message>
Modularize analysis, simplify Streamlit UI
Restructure analysis code into modular src packages and update the Streamlit app accordingly. Replaces src/kinetics.py with new modules (analysis, arrhenius, fitting, models, ode_systems) and adjusts imports throughout; introduces AnalysisResult/run_analysis interfaces. Refactors app.py: simpler UI, CSV support, template CSV download, consolidated RK4+least-squares workflow, updated plotting calls, and removed legacy options/metadata handling. Update README to reflect new methods and sample parameter changes (sample4 Ea/A), add regenerated sample_data and changes to generate_samples.py, and expand local .claude diagnostic commands. Removes verify_samples.py and updates reporter/plotting usages to match the new API.
</commit_message>
<xml_diff>
--- a/sample_data/sample4_multi_temp_arrhenius.xlsx
+++ b/sample_data/sample4_multi_temp_arrhenius.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>濃度_A (Concentration_A)
+          <t>涡度_A (Concentration_A)
 (mol/L)</t>
         </is>
       </c>
@@ -466,7 +466,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>備考 (Notes)
+          <t>備胝 (Notes)
 (-)</t>
         </is>
       </c>
@@ -483,7 +483,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>25.0°C 開始</t>
+          <t>25.0C start</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
         <v>10</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.214899</v>
+        <v>0.901007</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>25</v>
@@ -504,7 +504,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.046182</v>
+        <v>0.811814</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>25</v>
@@ -516,7 +516,7 @@
         <v>40</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.002133</v>
+        <v>0.659042</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>25</v>
@@ -528,7 +528,7 @@
         <v>60</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>9.8e-05</v>
+        <v>0.535019</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>25</v>
@@ -540,7 +540,7 @@
         <v>80</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>5e-06</v>
+        <v>0.434336</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>25</v>
@@ -552,7 +552,7 @@
         <v>100</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0</v>
+        <v>0.3526</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>25</v>
@@ -564,14 +564,14 @@
         <v>120</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0</v>
+        <v>0.286246</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>25</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>25.0°C 終了</t>
+          <t>25.0C end</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>35.0°C 開始</t>
+          <t>35.0C start</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.034297</v>
+        <v>0.818242</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>35</v>
@@ -608,7 +608,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.001176</v>
+        <v>0.669521</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>35</v>
@@ -620,7 +620,7 @@
         <v>40</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>1e-06</v>
+        <v>0.448258</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>35</v>
@@ -632,7 +632,7 @@
         <v>60</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0</v>
+        <v>0.300118</v>
       </c>
       <c r="C14" s="2" t="n">
         <v>35</v>
@@ -644,7 +644,7 @@
         <v>80</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.200935</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>35</v>
@@ -656,7 +656,7 @@
         <v>100</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>0</v>
+        <v>0.13453</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>35</v>
@@ -668,14 +668,14 @@
         <v>120</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>0</v>
+        <v>0.090071</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>35</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>35.0°C 終了</t>
+          <t>35.0C end</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>45.0°C 開始</t>
+          <t>45.0C start</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
         <v>10</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>0.000875</v>
+        <v>0.690421</v>
       </c>
       <c r="C19" s="2" t="n">
         <v>45</v>
@@ -712,7 +712,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>1e-06</v>
+        <v>0.476682</v>
       </c>
       <c r="C20" s="2" t="n">
         <v>45</v>
@@ -724,7 +724,7 @@
         <v>40</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>0</v>
+        <v>0.227225</v>
       </c>
       <c r="C21" s="2" t="n">
         <v>45</v>
@@ -736,7 +736,7 @@
         <v>60</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>0</v>
+        <v>0.108314</v>
       </c>
       <c r="C22" s="2" t="n">
         <v>45</v>
@@ -748,7 +748,7 @@
         <v>80</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>0</v>
+        <v>0.051631</v>
       </c>
       <c r="C23" s="2" t="n">
         <v>45</v>
@@ -760,7 +760,7 @@
         <v>100</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>0</v>
+        <v>0.024612</v>
       </c>
       <c r="C24" s="2" t="n">
         <v>45</v>
@@ -772,14 +772,14 @@
         <v>120</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>0</v>
+        <v>0.011732</v>
       </c>
       <c r="C25" s="2" t="n">
         <v>45</v>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>45.0°C 終了</t>
+          <t>45.0C end</t>
         </is>
       </c>
     </row>
@@ -795,7 +795,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>55.0°C 開始</t>
+          <t>55.0C start</t>
         </is>
       </c>
     </row>
@@ -804,7 +804,7 @@
         <v>10</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>1e-06</v>
+        <v>0.517352</v>
       </c>
       <c r="C27" s="2" t="n">
         <v>55</v>
@@ -816,7 +816,7 @@
         <v>20</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>0</v>
+        <v>0.267653</v>
       </c>
       <c r="C28" s="2" t="n">
         <v>55</v>
@@ -828,7 +828,7 @@
         <v>40</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>0</v>
+        <v>0.07163799999999999</v>
       </c>
       <c r="C29" s="2" t="n">
         <v>55</v>
@@ -840,7 +840,7 @@
         <v>60</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>0</v>
+        <v>0.019174</v>
       </c>
       <c r="C30" s="2" t="n">
         <v>55</v>
@@ -852,7 +852,7 @@
         <v>80</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>0</v>
+        <v>0.005132</v>
       </c>
       <c r="C31" s="2" t="n">
         <v>55</v>
@@ -864,7 +864,7 @@
         <v>100</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>0</v>
+        <v>0.001374</v>
       </c>
       <c r="C32" s="2" t="n">
         <v>55</v>
@@ -876,14 +876,14 @@
         <v>120</v>
       </c>
       <c r="B33" s="2" t="n">
-        <v>0</v>
+        <v>0.000368</v>
       </c>
       <c r="C33" s="2" t="n">
         <v>55</v>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>55.0°C 終了</t>
+          <t>55.0C end</t>
         </is>
       </c>
     </row>
@@ -919,7 +919,7 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>単位</t>
+          <t>单位</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>複数温度_Arrhenius_Ea=60kJ</t>
+          <t>multi_temp_Arrhenius_Ea=50kJ</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -944,7 +944,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>物質A</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr"/>
@@ -952,7 +952,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>初期濃度</t>
+          <t>初期涡度</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -972,7 +972,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>25-55°C</t>
+          <t>25-55C</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>テスト</t>
+          <t>test</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
@@ -1014,12 +1014,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>備考</t>
+          <t>備胝</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Ea=60kJ/mol, A=5e9</t>
+          <t>Ea=50kJ/mol, A=6e6</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>

</xml_diff>